<commit_message>
Fix contract staging Excel sheet
</commit_message>
<xml_diff>
--- a/docs/FLARE-contract-staging.xlsx
+++ b/docs/FLARE-contract-staging.xlsx
@@ -81,12 +81,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00B8860B"/>
+        <fgColor rgb="007A7A73"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="007A7A73"/>
+        <fgColor rgb="00B8860B"/>
       </patternFill>
     </fill>
     <fill>
@@ -142,14 +142,14 @@
     <xf numFmtId="0" fontId="7" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -520,7 +520,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
-    <col width="112" customWidth="1" min="2" max="2"/>
+    <col width="114" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -533,21 +533,21 @@
     <row r="4">
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Paste Copilot's three extraction tables into the matching data sheets, review, then grid-paste into SharePoint.</t>
+          <t>Paste Copilot's three extraction tables into the matching sheets, review, then grid-paste into SharePoint.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>What the contract PDFs populate</t>
+          <t>Column order matches Copilot's output</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Each contract fills ONE Contracts row, one-or-more ContractEntitlement rows (per path, per MDQ period), and — only if it has negotiated or discounted rates — one-or-more Rates rows (per component, per path, per window) with Contract filled. Shared RECOURSE rates are NOT in the contracts: load those into the Rates list from the pipelines' tariff sheets separately, with Contract left blank.</t>
+          <t>Each Copilot table ends with SourcePage and Flags, so those are the grey columns here — a straight paste from cell A lands every column in the right place, including the grey ones. The gold columns are NOT produced by Copilot; you fill them by hand (see below). They sit AFTER the grey columns so they never disturb the paste.</t>
         </is>
       </c>
     </row>
@@ -561,112 +561,112 @@
     <row r="10">
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Navy header  = loads into SharePoint. Paste these columns into the list.</t>
+          <t xml:space="preserve">  Navy = paste from Copilot, and loads into SharePoint.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Gold header  = loads too, but is a CONSTANT you fill down (RateBasis = Path for all negotiated transport rows).</t>
+          <t xml:space="preserve">  Grey = Copilot fills these too (SourcePage, Flags), but they are REVIEW ONLY — delete before loading.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Grey header  = review only. Do NOT paste into SharePoint — delete before loading.</t>
+          <t xml:space="preserve">  Gold = you fill by hand: SourcePDF after uploading the PDF; RateBasis = Path on every negotiated row.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Beige row    = worked example showing the expected format. Delete it before loading.</t>
+          <t xml:space="preserve">  Beige row = worked example. Delete it before loading.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Steps</t>
+          <t>Steps per contract (or small batch)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>1.  Run the Copilot extraction prompt (in the guide) on one contract, or a small batch, at a time.</t>
+          <t>1.  In M365 Copilot Chat, attach the contract PDF and run the extraction prompt (from the build guide).</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>2.  Paste TABLE 1 under Contracts, TABLE 2 under ContractEntitlement, TABLE 3 (if any) under Rates (negotiated).</t>
+          <t>2.  Copy each rendered table (use the table's copy control, not the raw text) and paste under the headers:</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="B18" s="8" t="inlineStr">
-        <is>
-          <t>3.  REVIEW every number and date against the page in the SourcePage column. The one step you can't skip.</t>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      TABLE 1 -&gt; Contracts,  TABLE 2 -&gt; ContractEntitlement,  TABLE 3 (if any) -&gt; Rates (negotiated).</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>4.  Confirm Pipeline / RateSchedule / Path spellings EXACTLY match your dimension-list Titles, or the lookup imports blank.</t>
+      <c r="B19" s="8" t="inlineStr">
+        <is>
+          <t>3.  REVIEW every number and date against its SourcePage cell. The one step you can't skip.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>5.  On the Rates sheet, fill RateBasis = Path down every row (all negotiated transport rates are path-based).</t>
+          <t>4.  Fill the gold columns: SourcePDF (after upload) on Contracts; RateBasis = Path on every Rates row.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>6.  Delete the example row and the grey review-only columns.</t>
+          <t>5.  Confirm Pipeline / RateSchedule / Path spellings exactly match your dimension-list Titles.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>7.  Grid-paste in load order: Contracts -&gt; ContractEntitlement -&gt; Rates (negotiated).</t>
+          <t>6.  Delete the example row and the grey columns, then grid-paste in order: Contracts -&gt; ContractEntitlement -&gt; Rates (negotiated).</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>Loading the Rates (negotiated) sheet</t>
+          <t>If a paste lands everything in one column</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>These rows load into the SAME Rates list as your recourse rates, but with Contract filled and RateType = Negotiated/Discount. Leave the list's Point column blank for these (they're path-based), and set SourceRef (the agreement link) after you upload the PDFs. RateType tells them apart from the Contract-blank recourse rows.</t>
+          <t>That happens when you copied the raw pipe text instead of the rendered table. Either re-copy the rendered table, or select the mashed column and use Data -&gt; Text to Columns with delimiter = | (pipe).</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>Lookup-matching reminder</t>
+          <t>Loading the Rates (negotiated) rows</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>On ContractEntitlement and Rates, the Contract column must contain the ContractID text exactly as it appears in the Contracts list Title. Path must match the Paths list Title. SharePoint links lookups by matching that text.</t>
+          <t>They load into the SAME Rates list as recourse rates, but with Contract filled and RateType = Negotiated/Discount. Leave the list's Point column blank (path-based), and set SourceRef after uploading the agreement.</t>
         </is>
       </c>
     </row>
@@ -691,9 +691,9 @@
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="30" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
-    <col width="24" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="26" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -732,71 +732,71 @@
           <t>TermEnd</t>
         </is>
       </c>
-      <c r="H1" s="9" t="inlineStr">
-        <is>
-          <t>SourcePDF</t>
+      <c r="H1" s="10" t="inlineStr">
+        <is>
+          <t>SourcePage  (review)</t>
         </is>
       </c>
       <c r="I1" s="10" t="inlineStr">
         <is>
-          <t>SourcePage  (review only)</t>
-        </is>
-      </c>
-      <c r="J1" s="10" t="inlineStr">
-        <is>
-          <t>Flags  (review only)</t>
+          <t>Flags  (review)</t>
+        </is>
+      </c>
+      <c r="J1" s="11" t="inlineStr">
+        <is>
+          <t>SourcePDF  (fill after upload)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="11" t="inlineStr">
+      <c r="A2" s="12" t="inlineStr">
         <is>
           <t>GTN-1234</t>
         </is>
       </c>
-      <c r="B2" s="11" t="inlineStr">
+      <c r="B2" s="12" t="inlineStr">
         <is>
           <t>Acme Energy Marketing</t>
         </is>
       </c>
-      <c r="C2" s="11" t="inlineStr">
+      <c r="C2" s="12" t="inlineStr">
         <is>
           <t>GTN</t>
         </is>
       </c>
-      <c r="D2" s="11" t="inlineStr">
+      <c r="D2" s="12" t="inlineStr">
         <is>
           <t>FT-1</t>
         </is>
       </c>
-      <c r="E2" s="11" t="inlineStr">
+      <c r="E2" s="12" t="inlineStr">
         <is>
           <t>Shaped</t>
         </is>
       </c>
-      <c r="F2" s="11" t="inlineStr">
+      <c r="F2" s="12" t="inlineStr">
         <is>
           <t>2024-11-01</t>
         </is>
       </c>
-      <c r="G2" s="11" t="inlineStr">
+      <c r="G2" s="12" t="inlineStr">
         <is>
           <t>2029-10-31</t>
         </is>
       </c>
-      <c r="H2" s="11" t="inlineStr">
-        <is>
-          <t>(paste library link after upload)</t>
-        </is>
-      </c>
-      <c r="I2" s="11" t="inlineStr">
+      <c r="H2" s="12" t="inlineStr">
         <is>
           <t>p.1, Exh. A p.7</t>
         </is>
       </c>
-      <c r="J2" s="11" t="inlineStr">
+      <c r="I2" s="12" t="inlineStr">
         <is>
           <t>MDQ shape on Exhibit A</t>
+        </is>
+      </c>
+      <c r="J2" s="12" t="inlineStr">
+        <is>
+          <t>(library link)</t>
         </is>
       </c>
     </row>
@@ -820,9 +820,9 @@
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -856,66 +856,66 @@
           <t>EffectiveEnd</t>
         </is>
       </c>
-      <c r="G1" s="9" t="inlineStr">
+      <c r="G1" s="10" t="inlineStr">
+        <is>
+          <t>SourcePage  (review)</t>
+        </is>
+      </c>
+      <c r="H1" s="10" t="inlineStr">
+        <is>
+          <t>Flags  (review)</t>
+        </is>
+      </c>
+      <c r="I1" s="9" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="H1" s="10" t="inlineStr">
-        <is>
-          <t>SourcePage  (review only)</t>
-        </is>
-      </c>
-      <c r="I1" s="10" t="inlineStr">
-        <is>
-          <t>Flags  (review only)</t>
-        </is>
-      </c>
     </row>
     <row r="2">
-      <c r="A2" s="11" t="inlineStr">
+      <c r="A2" s="12" t="inlineStr">
         <is>
           <t>GTN-1234 KGT-Malin 2024-11</t>
         </is>
       </c>
-      <c r="B2" s="11" t="inlineStr">
+      <c r="B2" s="12" t="inlineStr">
         <is>
           <t>GTN-1234</t>
         </is>
       </c>
-      <c r="C2" s="11" t="inlineStr">
+      <c r="C2" s="12" t="inlineStr">
         <is>
           <t>GTN Kingsgate-Malin</t>
         </is>
       </c>
-      <c r="D2" s="11" t="inlineStr">
+      <c r="D2" s="12" t="inlineStr">
         <is>
           <t>50000</t>
         </is>
       </c>
-      <c r="E2" s="11" t="inlineStr">
+      <c r="E2" s="12" t="inlineStr">
         <is>
           <t>2024-11-01</t>
         </is>
       </c>
-      <c r="F2" s="11" t="inlineStr">
+      <c r="F2" s="12" t="inlineStr">
         <is>
           <t>2025-03-31</t>
         </is>
       </c>
-      <c r="G2" s="11" t="inlineStr">
+      <c r="G2" s="12" t="inlineStr">
+        <is>
+          <t>Exh. A p.7</t>
+        </is>
+      </c>
+      <c r="H2" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I2" s="12" t="inlineStr">
         <is>
           <t>Winter shape</t>
-        </is>
-      </c>
-      <c r="H2" s="11" t="inlineStr">
-        <is>
-          <t>Exh. A p.7</t>
-        </is>
-      </c>
-      <c r="I2" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
         </is>
       </c>
     </row>
@@ -939,14 +939,14 @@
     <col width="24" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="17" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
     <col width="15" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
     <col width="15" customWidth="1" min="11" max="11"/>
-    <col width="16" customWidth="1" min="12" max="12"/>
-    <col width="20" customWidth="1" min="13" max="13"/>
-    <col width="26" customWidth="1" min="14" max="14"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
+    <col width="22" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -1005,87 +1005,87 @@
           <t>EffectiveEnd</t>
         </is>
       </c>
-      <c r="L1" s="12" t="inlineStr">
+      <c r="L1" s="10" t="inlineStr">
+        <is>
+          <t>SourcePage  (review)</t>
+        </is>
+      </c>
+      <c r="M1" s="10" t="inlineStr">
+        <is>
+          <t>Flags  (review)</t>
+        </is>
+      </c>
+      <c r="N1" s="11" t="inlineStr">
         <is>
           <t>RateBasis  (= Path)</t>
         </is>
       </c>
-      <c r="M1" s="10" t="inlineStr">
-        <is>
-          <t>SourcePage  (review only)</t>
-        </is>
-      </c>
-      <c r="N1" s="10" t="inlineStr">
-        <is>
-          <t>Flags  (review only)</t>
-        </is>
-      </c>
     </row>
     <row r="2">
-      <c r="A2" s="11" t="inlineStr">
+      <c r="A2" s="12" t="inlineStr">
         <is>
           <t>GTN-1234 KGT-Malin reservation</t>
         </is>
       </c>
-      <c r="B2" s="11" t="inlineStr">
+      <c r="B2" s="12" t="inlineStr">
         <is>
           <t>GTN-1234</t>
         </is>
       </c>
-      <c r="C2" s="11" t="inlineStr">
+      <c r="C2" s="12" t="inlineStr">
         <is>
           <t>FT-1</t>
         </is>
       </c>
-      <c r="D2" s="11" t="inlineStr">
+      <c r="D2" s="12" t="inlineStr">
         <is>
           <t>GTN Kingsgate-Malin</t>
         </is>
       </c>
-      <c r="E2" s="11" t="inlineStr">
+      <c r="E2" s="12" t="inlineStr">
         <is>
           <t>Negotiated</t>
         </is>
       </c>
-      <c r="F2" s="11" t="inlineStr">
+      <c r="F2" s="12" t="inlineStr">
         <is>
           <t>Reservation</t>
         </is>
       </c>
-      <c r="G2" s="11" t="inlineStr"/>
-      <c r="H2" s="11" t="inlineStr">
+      <c r="G2" s="12" t="inlineStr"/>
+      <c r="H2" s="12" t="inlineStr">
         <is>
           <t>0.30</t>
         </is>
       </c>
-      <c r="I2" s="11" t="inlineStr">
+      <c r="I2" s="12" t="inlineStr">
         <is>
           <t>$/Dth/month</t>
         </is>
       </c>
-      <c r="J2" s="11" t="inlineStr">
+      <c r="J2" s="12" t="inlineStr">
         <is>
           <t>2024-11-01</t>
         </is>
       </c>
-      <c r="K2" s="11" t="inlineStr">
+      <c r="K2" s="12" t="inlineStr">
         <is>
           <t>2029-10-31</t>
         </is>
       </c>
-      <c r="L2" s="11" t="inlineStr">
+      <c r="L2" s="12" t="inlineStr">
+        <is>
+          <t>Exh. B p.9</t>
+        </is>
+      </c>
+      <c r="M2" s="12" t="inlineStr">
+        <is>
+          <t>fuel stays recourse</t>
+        </is>
+      </c>
+      <c r="N2" s="12" t="inlineStr">
         <is>
           <t>Path</t>
-        </is>
-      </c>
-      <c r="M2" s="11" t="inlineStr">
-        <is>
-          <t>Exh. B p.9</t>
-        </is>
-      </c>
-      <c r="N2" s="11" t="inlineStr">
-        <is>
-          <t>negotiated reservation; fuel stays recourse</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update pipeline rate database setup plan and contract staging Excel sheet
</commit_message>
<xml_diff>
--- a/docs/FLARE-contract-staging.xlsx
+++ b/docs/FLARE-contract-staging.xlsx
@@ -11,6 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contracts" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ContractEntitlement" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rates (negotiated)" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rates (recourse)" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -516,7 +517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:B28"/>
+  <dimension ref="B2:B24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -526,28 +527,28 @@
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>FLARE — contract staging workbook</t>
+          <t>FLARE — contract &amp; tariff staging workbook</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Paste Copilot's three extraction tables into the matching sheets, review, then grid-paste into SharePoint.</t>
+          <t>Paste Copilot's extraction tables into the matching sheets, review, then grid-paste into SharePoint.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Column order matches Copilot's output</t>
+          <t>The two rate sources</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Each Copilot table ends with SourcePage and Flags, so those are the grey columns here — a straight paste from cell A lands every column in the right place, including the grey ones. The gold columns are NOT produced by Copilot; you fill them by hand (see below). They sit AFTER the grey columns so they never disturb the paste.</t>
+          <t>CONTRACTS give you: one Contracts row, its ContractEntitlement rows, and — only if the deal is negotiated/discounted — Rates (negotiated) rows with Contract FILLED. TARIFF SHEETS give you the shared recourse curve: Rates (recourse) rows with Contract BLANK. Both Rates sheets load into the SAME Rates list; the Contract column is what tells them apart.</t>
         </is>
       </c>
     </row>
@@ -575,7 +576,7 @@
     <row r="12">
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Gold = you fill by hand: SourcePDF after uploading the PDF; RateBasis = Path on every negotiated row.</t>
+          <t xml:space="preserve">  Gold = you fill by hand: SourcePDF (after upload), RateBasis = Path (negotiated), RateType = Recourse (recourse).</t>
         </is>
       </c>
     </row>
@@ -589,84 +590,63 @@
     <row r="15">
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Steps per contract (or small batch)</t>
+          <t>Steps</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>1.  In M365 Copilot Chat, attach the contract PDF and run the extraction prompt (from the build guide).</t>
+          <t>1.  CONTRACTS: run the contract extraction prompt with a contract PDF attached; paste TABLE 1 -&gt; Contracts, TABLE 2 -&gt; ContractEntitlement, TABLE 3 (if any) -&gt; Rates (negotiated).</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>2.  Copy each rendered table (use the table's copy control, not the raw text) and paste under the headers:</t>
+          <t>2.  TARIFF: run the recourse extraction prompt with a pipeline's Statement of Effective Rates attached; paste the result -&gt; Rates (recourse).</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">      TABLE 1 -&gt; Contracts,  TABLE 2 -&gt; ContractEntitlement,  TABLE 3 (if any) -&gt; Rates (negotiated).</t>
+      <c r="B18" s="8" t="inlineStr">
+        <is>
+          <t>3.  REVIEW every number and date against its SourcePage cell. The one step you can't skip.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="B19" s="8" t="inlineStr">
-        <is>
-          <t>3.  REVIEW every number and date against its SourcePage cell. The one step you can't skip.</t>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>4.  Fill the gold columns: SourcePDF (Contracts); RateBasis = Path (Rates negotiated); RateType = Recourse (Rates recourse).</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>4.  Fill the gold columns: SourcePDF (after upload) on Contracts; RateBasis = Path on every Rates row.</t>
+          <t>5.  Confirm RateSchedule / Path spellings exactly match your dimension-list Titles.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>5.  Confirm Pipeline / RateSchedule / Path spellings exactly match your dimension-list Titles.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>6.  Delete the example row and the grey columns, then grid-paste in order: Contracts -&gt; ContractEntitlement -&gt; Rates (negotiated).</t>
+          <t>6.  Delete the example row and grey columns, then grid-paste. Recourse rows can load once RateSchedules and Paths exist; negotiated rows need Contracts loaded first.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Loading the two Rates sheets</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="B24" s="3" t="inlineStr">
-        <is>
-          <t>If a paste lands everything in one column</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>That happens when you copied the raw pipe text instead of the rendered table. Either re-copy the rendered table, or select the mashed column and use Data -&gt; Text to Columns with delimiter = | (pipe).</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="B27" s="3" t="inlineStr">
-        <is>
-          <t>Loading the Rates (negotiated) rows</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="B28" s="2" t="inlineStr">
-        <is>
-          <t>They load into the SAME Rates list as recourse rates, but with Contract filled and RateType = Negotiated/Discount. Leave the list's Point column blank (path-based), and set SourceRef after uploading the agreement.</t>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Both go into the Rates list. RECOURSE rows: Contract blank, RateType = Recourse, Point blank. NEGOTIATED rows: Contract filled, RateType = Negotiated/Discount, Point blank (path-based). Set SourceRef (the tariff sheet or agreement link) after upload. If a paste lands in one column, copy the rendered table (not raw text), or use Data -&gt; Text to Columns with delimiter = | (pipe).</t>
         </is>
       </c>
     </row>
@@ -766,7 +746,7 @@
       </c>
       <c r="D2" s="12" t="inlineStr">
         <is>
-          <t>FT-1</t>
+          <t>GTN FTS-1</t>
         </is>
       </c>
       <c r="E2" s="12" t="inlineStr">
@@ -1034,7 +1014,7 @@
       </c>
       <c r="C2" s="12" t="inlineStr">
         <is>
-          <t>FT-1</t>
+          <t>GTN FTS-1</t>
         </is>
       </c>
       <c r="D2" s="12" t="inlineStr">
@@ -1086,6 +1066,161 @@
       <c r="N2" s="12" t="inlineStr">
         <is>
           <t>Path</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="18" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="9" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="B1" s="9" t="inlineStr">
+        <is>
+          <t>RateSchedule</t>
+        </is>
+      </c>
+      <c r="C1" s="9" t="inlineStr">
+        <is>
+          <t>Path</t>
+        </is>
+      </c>
+      <c r="D1" s="9" t="inlineStr">
+        <is>
+          <t>RateBasis</t>
+        </is>
+      </c>
+      <c r="E1" s="9" t="inlineStr">
+        <is>
+          <t>Component</t>
+        </is>
+      </c>
+      <c r="F1" s="9" t="inlineStr">
+        <is>
+          <t>ComponentDetail</t>
+        </is>
+      </c>
+      <c r="G1" s="9" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="H1" s="9" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="I1" s="9" t="inlineStr">
+        <is>
+          <t>EffectiveStart</t>
+        </is>
+      </c>
+      <c r="J1" s="9" t="inlineStr">
+        <is>
+          <t>EffectiveEnd</t>
+        </is>
+      </c>
+      <c r="K1" s="10" t="inlineStr">
+        <is>
+          <t>SourcePage  (review)</t>
+        </is>
+      </c>
+      <c r="L1" s="10" t="inlineStr">
+        <is>
+          <t>Flags  (review)</t>
+        </is>
+      </c>
+      <c r="M1" s="11" t="inlineStr">
+        <is>
+          <t>RateType  (= Recourse)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="12" t="inlineStr">
+        <is>
+          <t>GTN FTS-1 KGT-Malin reservation</t>
+        </is>
+      </c>
+      <c r="B2" s="12" t="inlineStr">
+        <is>
+          <t>GTN FTS-1</t>
+        </is>
+      </c>
+      <c r="C2" s="12" t="inlineStr">
+        <is>
+          <t>GTN Kingsgate-Malin</t>
+        </is>
+      </c>
+      <c r="D2" s="12" t="inlineStr">
+        <is>
+          <t>Path</t>
+        </is>
+      </c>
+      <c r="E2" s="12" t="inlineStr">
+        <is>
+          <t>Reservation</t>
+        </is>
+      </c>
+      <c r="F2" s="12" t="inlineStr"/>
+      <c r="G2" s="12" t="inlineStr">
+        <is>
+          <t>0.4200</t>
+        </is>
+      </c>
+      <c r="H2" s="12" t="inlineStr">
+        <is>
+          <t>$/Dth/month</t>
+        </is>
+      </c>
+      <c r="I2" s="12" t="inlineStr">
+        <is>
+          <t>2024-01-01</t>
+        </is>
+      </c>
+      <c r="J2" s="12" t="inlineStr"/>
+      <c r="K2" s="12" t="inlineStr">
+        <is>
+          <t>Eff. Rates Sheet 5</t>
+        </is>
+      </c>
+      <c r="L2" s="12" t="inlineStr">
+        <is>
+          <t>max recourse</t>
+        </is>
+      </c>
+      <c r="M2" s="12" t="inlineStr">
+        <is>
+          <t>Recourse</t>
         </is>
       </c>
     </row>

</xml_diff>